<commit_message>
productores.xlsx: Curuca es comprador, no productor (nota en la ficha)
Gonzalo 18/09/2026: Curuca revende fruta de otros. Por eso en el Plan de
Cargas sus camiones figuran con el nombre del productor real y no se
pueden cruzar con la planilla de cargas 2026 (Curuca aparece solo en dos
cargas canceladas). La nota deja las carpetas de Etimex donde esta el
vendedor exacto de cada camion. CARGAS_JSON regenerado (paso 5h).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/productores.xlsx
+++ b/fuentes/productores.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="237">
   <si>
     <t>Productor</t>
   </si>
@@ -462,6 +462,9 @@
   </si>
   <si>
     <t>Curuca</t>
+  </si>
+  <si>
+    <t>COMPRADOR, no productor (Gonzalo 18/09/2026): revende fruta de otros. En el Plan de Cargas sus camiones figuran con el nombre del productor real (Curuca solo aparece 2 veces, canceladas: 27/02 y 24/03/2026). Compras 2026: sem 5 con FG (carpeta BRB011-26) y sem 14-16 con Chabat/Etimex (carpetas BRB029-26, BRB035-26, BRB036-26); el vendedor exacto de cada camion esta en esas carpetas de Etimex.</t>
   </si>
   <si>
     <t>Furlani</t>
@@ -1902,6 +1905,9 @@
       </c>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
+      <c r="J14" s="0" t="s">
+        <v>127</v>
+      </c>
       <c r="K14" s="3">
         <v>6</v>
       </c>
@@ -1919,10 +1925,10 @@
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C15" s="0" t="s">
         <v>25</v>
@@ -1931,10 +1937,10 @@
         <v>26</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G15" s="3">
         <v>-26.709688</v>
@@ -1949,7 +1955,7 @@
         <v>11.5</v>
       </c>
       <c r="M15" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="O15" s="0">
         <v>33000</v>
@@ -1958,25 +1964,25 @@
         <v>31</v>
       </c>
       <c r="S15" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T15" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="U15" s="6"/>
       <c r="V15" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="W15" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C16" s="0" t="s">
         <v>25</v>
@@ -1994,16 +2000,16 @@
         <v>-48.876062</v>
       </c>
       <c r="J16" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K16" s="3">
         <v>17</v>
       </c>
       <c r="L16" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="M16" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O16" s="0">
         <v>85000</v>
@@ -2012,25 +2018,25 @@
         <v>31</v>
       </c>
       <c r="S16" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="T16" s="6" t="s">
         <v>94</v>
       </c>
       <c r="U16" s="6"/>
       <c r="V16" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="W16" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C17" s="0" t="s">
         <v>25</v>
@@ -2042,40 +2048,40 @@
         <v>66</v>
       </c>
       <c r="J17" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="K17" s="0">
         <v>8</v>
       </c>
       <c r="L17" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="M17" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="P17" s="0" t="s">
         <v>31</v>
       </c>
       <c r="S17" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="T17" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="U17" s="6"/>
       <c r="V17" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="W17" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C18" s="0" t="s">
         <v>25</v>
@@ -2087,7 +2093,7 @@
         <v>46</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G18" s="0">
         <v>-26.6724542</v>
@@ -2096,34 +2102,34 @@
         <v>-48.9256154</v>
       </c>
       <c r="J18" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K18" s="0">
         <v>4</v>
       </c>
       <c r="L18" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="P18" s="0" t="s">
         <v>31</v>
       </c>
       <c r="S18" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="T18" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="U18" s="6"/>
       <c r="V18" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="W18" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C19" s="0" t="s">
         <v>25</v>
@@ -2141,23 +2147,23 @@
         <v>-48.850312</v>
       </c>
       <c r="J19" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K19" s="0">
         <v>1.5</v>
       </c>
       <c r="M19" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="P19" s="0" t="s">
         <v>31</v>
       </c>
       <c r="T19" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="U19" s="6"/>
       <c r="V19" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="W19" s="6" t="s">
         <v>111</v>
@@ -2165,19 +2171,19 @@
     </row>
     <row r="20">
       <c r="A20" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D20" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G20" s="0">
         <v>-25.3264</v>
@@ -2186,19 +2192,19 @@
         <v>-55.3721</v>
       </c>
       <c r="J20" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K20" s="0">
         <v>65</v>
       </c>
       <c r="L20" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="M20" s="0" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T20" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="V20" s="0">
         <v>1388</v>
@@ -2209,16 +2215,16 @@
     </row>
     <row r="21">
       <c r="A21" s="0" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C21" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D21" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G21" s="0">
         <v>-25.34481</v>
@@ -2227,19 +2233,19 @@
         <v>-55.48031</v>
       </c>
       <c r="J21" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="K21" s="0">
         <v>15</v>
       </c>
       <c r="L21" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="M21" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T21" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="V21" s="0">
         <v>1402</v>
@@ -2250,111 +2256,111 @@
     </row>
     <row r="22">
       <c r="A22" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J22" s="0" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K22" s="0">
         <v>0</v>
       </c>
       <c r="T22" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J23" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K23" s="0">
         <v>17</v>
       </c>
       <c r="L23" s="0" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="T23" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J24" s="0" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K24" s="0">
         <v>11</v>
       </c>
       <c r="L24" s="0" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="T24" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J25" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K25" s="0">
         <v>7</v>
       </c>
       <c r="L25" s="0" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="T25" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J26" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="K26" s="0">
         <v>0</v>
       </c>
       <c r="T26" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -2375,202 +2381,202 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="0" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="0" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="0" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="0" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fichas: notas de procedencia vaciadas (salvo Curuca) y fotos de packing de Paraguay HF en las fichas (sesion peer, 24/09)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/productores.xlsx
+++ b/fuentes/productores.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\poronga\fuentes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\PorongaEnLaNube\gonza_pepe\fuentes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A4F4A7-A7E6-49C4-B837-32982C629939}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57F4B821-81A0-4280-8A72-2073E2E93BA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{0F9C3186-219F-4CB3-AD9B-1236109C1198}"/>
   </bookViews>
@@ -17,9 +17,9 @@
     <sheet name="como_llenar" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'productores'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">productores!$A$1:$K$1</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="217">
   <si>
     <t>Productor</t>
   </si>
@@ -170,9 +170,6 @@
     <t>Bomplandt</t>
   </si>
   <si>
-    <t>Contacto (WhatsApp): dato de Gonzalo 09/09/2026.</t>
-  </si>
-  <si>
     <t>Estrada Bomplandt, S/N, Bairro Bomplandt</t>
   </si>
   <si>
@@ -227,9 +224,6 @@
     <t>Braco Miguel (dato anterior, sin verificar)</t>
   </si>
   <si>
-    <t>Direccion y Plus code 84F4+3Q decodificado a coordenadas (Gonzalo 09/09/2026), precision ~125 m. | Contacto (WhatsApp): dato de Gonzalo 09/09/2026.</t>
-  </si>
-  <si>
     <t>Valdemar Tuti</t>
   </si>
   <si>
@@ -257,9 +251,6 @@
     <t>Araquari / SC</t>
   </si>
   <si>
-    <t>Ubicacion y pies: dato de Gonzalo 08/09/2026. Antes figuraba Guaramirim; el punto cae en Araquari, en el limite entre los dos. | Pies de banana corregidos a 65.000 (antes 90.000) y variedad Caturra / Grande Naine: dato de Gonzalo 09/09/2026. | Contacto (WhatsApp): dato de Gonzalo 09/09/2026.</t>
-  </si>
-  <si>
     <t>Plus code G33W+GCQ (Araquari, SC)</t>
   </si>
   <si>
@@ -284,9 +275,6 @@
     <t>Barra Velha / SC</t>
   </si>
   <si>
-    <t>Ubicacion: Plus code 585H867C+VJ decodificado a coordenadas (Gonzalo 09/09/2026), precision ~125 m.</t>
-  </si>
-  <si>
     <t>Jhony Viera</t>
   </si>
   <si>
@@ -311,9 +299,6 @@
     <t>Agro curupa; Corupá; Corupa</t>
   </si>
   <si>
-    <t>Ubicacion: coordenadas y Plus code 8558+578, dato de Gonzalo 09/09/2026.</t>
-  </si>
-  <si>
     <t>Plus code 8558+578 (Luiz Alves, SC)</t>
   </si>
   <si>
@@ -332,9 +317,6 @@
     <t>Lagoinha</t>
   </si>
   <si>
-    <t>Contacto (WhatsApp): dato de Gonzalo 09/09/2026. | Ubicación pasada por Gonzalo 10/09/2026: cerca de São João do Itaperiú, CEP 88395-000, Plus code 585HC5H4+FXG (-26.5713010, -48.8425407)</t>
-  </si>
-  <si>
     <t>+55 47 9960-1575</t>
   </si>
   <si>
@@ -353,9 +335,6 @@
     <t>Ivo; Ivo Zimerman</t>
   </si>
   <si>
-    <t>Ubicacion: dato de Gonzalo 09/09/2026 (coordenadas + Plus code 84W9+6RX Luiz Alves). Antes figuraba municipio "brazo miguel sc" y sin coordenadas. Pies de banana: 35.000, dato de Gonzalo 09/09/2026. Hectareas de banana: 10, va a plantar mas (Gonzalo 09/09/2026). | Contacto (WhatsApp): dato de Gonzalo 09/09/2026.</t>
-  </si>
-  <si>
     <t>Ivo Zimerman</t>
   </si>
   <si>
@@ -407,9 +386,6 @@
     <t>Baixo Canoas</t>
   </si>
   <si>
-    <t>Contacto (WhatsApp): dato de Gonzalo 09/09/2026. | Ubicación pasada por Gonzalo 10/09/2026: Plus code 585H75M7+99H (-26.7165700, -48.8365060), zona Baixo Canoas</t>
-  </si>
-  <si>
     <t>Wagner Schveitzer</t>
   </si>
   <si>
@@ -443,9 +419,6 @@
     <t>Sao Braz</t>
   </si>
   <si>
-    <t>Contacto (WhatsApp): dato de Gonzalo 09/09/2026. | Direccion y Plus code 768J+GH decodificado a coordenadas (Gonzalo 09/09/2026), precision ~125 m.</t>
-  </si>
-  <si>
     <t>Sergio Correa</t>
   </si>
   <si>
@@ -464,9 +437,6 @@
     <t>Curuca</t>
   </si>
   <si>
-    <t>COMPRADOR, no productor (Gonzalo 18/09/2026): revende fruta de otros. En el Plan de Cargas sus camiones figuran con el nombre del productor real (Curuca solo aparece 2 veces, canceladas: 27/02 y 24/03/2026). Compras 2026: sem 5 con FG (carpeta BRB011-26) y sem 14-16 con Chabat/Etimex (carpetas BRB029-26, BRB035-26, BRB036-26); el vendedor exacto de cada camion esta en esas carpetas de Etimex.</t>
-  </si>
-  <si>
     <t>Furlani</t>
   </si>
   <si>
@@ -500,9 +470,6 @@
     <t>Osnildo Stein</t>
   </si>
   <si>
-    <t>Ubicacion (municipio y CEP, sin coordenadas) y pies de banana: 85.000, dato de Gonzalo 09/09/2026. Coordenadas decodificadas del Plus code 84MF+4H (Gonzalo 09/09/2026), precision ~125 m. | Contacto (WhatsApp): dato de Gonzalo 09/09/2026.</t>
-  </si>
-  <si>
     <t>Plus code 84MF+4H (Luiz Alves, SC, CEP 89115-000)</t>
   </si>
   <si>
@@ -521,9 +488,6 @@
     <t>Josemar Provesi</t>
   </si>
   <si>
-    <t>Direccion (sin coordenadas): dato de Gonzalo 09/09/2026. | Contacto (WhatsApp): dato de Gonzalo 09/09/2026.</t>
-  </si>
-  <si>
     <t>Estrada Geral Rio Novo, 9500, Barra Velha, SC</t>
   </si>
   <si>
@@ -548,9 +512,6 @@
     <t>Estr. Braço Alberto (cerca)</t>
   </si>
   <si>
-    <t>Contacto (WhatsApp): dato de Gonzalo 09/09/2026. | Ubicación pasada por Gonzalo 10/09/2026: cerca de Estr. Braço Alberto, Luiz Alves, Plus code 585H83HF+2Q6 (-26.6724542, -48.9256154)</t>
-  </si>
-  <si>
     <t>Maikon Zappellini</t>
   </si>
   <si>
@@ -563,9 +524,6 @@
     <t>Shapo</t>
   </si>
   <si>
-    <t>Ubicacion: Plus code 585H947X+PV decodificado a coordenadas (Gonzalo 09/09/2026), precision ~125 m; vecino de Ivo y Stein.</t>
-  </si>
-  <si>
     <t>Plus code 947X+9Q / 585H947X+PV (Luiz Alves, SC, CEP 89115-000)</t>
   </si>
   <si>
@@ -587,9 +545,6 @@
     <t>Tembiapora / Caaguazu</t>
   </si>
   <si>
-    <t>Ubicacion: plus code pasado por Gonzalo 13/09/2026. Lote visto en origen ese dia: corte 5, calibre 38-42 (30-33 mm), pulpa 21,2 C, llenado corto, pitting en cascara, fruta manipulada mojada; ver guia de corte hoja 7. | Km por ruta OSRM 15/09/2026 desde las coordenadas de la ficha. Plan de Cargas: 120 camiones desde ene/2024 (39 en 2024, 16 en 2025, 65 en 2026), ~977 cajas/camion, TT mediana 4 dias. | Nombre_completo = exportador que figura en el Plan de Cargas (43 cargas 2026); confirmar si es el productor o su empresa.</t>
-  </si>
-  <si>
     <t>Hugo Franco</t>
   </si>
   <si>
@@ -605,9 +560,6 @@
     <t>MS; PY MS</t>
   </si>
   <si>
-    <t>Ubicacion: plus code 5866MG49+3V pasado por Gonzalo 10/09/2026 (precision ~14 m); visita el 11/09/2026. Por coordenadas caeria en el distrito Raul Arsenio Oviedo, sin confirmar. Plan de Cargas: frontera Salto, transportista Lider Express, ~980 cajas/camion, TT mediana 4 dias, 115 camiones desde ene/2024 (84 en 2024, 16 en 2025, 15 en 2026 jun-set). Km por ruta OSRM 15/09/2026. | Nombre_completo = exportador que figura en el Plan de Cargas (en 2 cargas figura Emprendimientos Karen); transportistas G.S.C.S. Paraguay Ttes. y Lider Express.</t>
-  </si>
-  <si>
     <t>Milciades Sosa</t>
   </si>
   <si>
@@ -620,18 +572,12 @@
     <t>EC; PY EC</t>
   </si>
   <si>
-    <t>Plan de Cargas: 88 camiones (78 en 2024, 10 en 2025), sin cargas en 2026; ~936 cajas/camion, TT mediana 4 dias. Ubicacion, hectareas y contacto: a cargar.</t>
-  </si>
-  <si>
     <t>Paraguay DF</t>
   </si>
   <si>
     <t>DF; PY DF</t>
   </si>
   <si>
-    <t>Plan de Cargas: 70 camiones (40 en 2024, 13 en 2025, 17 en 2026), ~981 cajas/camion, TT mediana 4 dias. Ubicacion, hectareas y contacto: a cargar. | Nombre_completo = exportador que figura en el Plan de Cargas; transportista habitual Compass (Jauser en set/2026).</t>
-  </si>
-  <si>
     <t>Diego Fernandez</t>
   </si>
   <si>
@@ -641,9 +587,6 @@
     <t>GM; PY GM</t>
   </si>
   <si>
-    <t>Plan de Cargas: 42 camiones (25 en 2024, 6 en 2025, 11 en 2026), ~972 cajas/camion, TT mediana 5 dias; faltantes acumulados 508 cajas, el mas alto de Paraguay: revisar. Ubicacion, hectareas y contacto: a cargar. | Nombre_completo = exportador que figura en el Plan de Cargas (parece empresa, no persona); transportistas Surcentral y Lider Express.</t>
-  </si>
-  <si>
     <t>Servi Fel (Servifel)</t>
   </si>
   <si>
@@ -653,9 +596,6 @@
     <t>AS; PY AS</t>
   </si>
   <si>
-    <t>Plan de Cargas: productor nuevo, 7 camiones desde el 11/08/2026, ~980 cajas/camion, TT mediana 3 dias. Ubicacion, hectareas y contacto: a cargar. | Nombre_completo = exportador que figura en el Plan de Cargas; transportista Marso Emprendimientos S.R.L. (set/2026).</t>
-  </si>
-  <si>
     <t>Alvaro Saldivar</t>
   </si>
   <si>
@@ -668,9 +608,6 @@
     <t>SF; PY SF</t>
   </si>
   <si>
-    <t>Plan de Cargas: un solo camion, el 27/02/2024. Ubicacion, hectareas y contacto: a cargar.</t>
-  </si>
-  <si>
     <t>feb 2024</t>
   </si>
   <si>
@@ -683,13 +620,13 @@
     <t>un productor nuevo o si cambia algo.</t>
   </si>
   <si>
-    <t xml:space="preserve">Productor  = nombre canonico. NO tocar los que ya estan: son los que el</t>
+    <t>Productor  = nombre canonico. NO tocar los que ya estan: son los que el</t>
   </si>
   <si>
     <t xml:space="preserve">             script ya reconoce.</t>
   </si>
   <si>
-    <t xml:space="preserve">Alias      = todas las formas en que lo escribis en "cargas 2026.xlsx"</t>
+    <t>Alias      = todas las formas en que lo escribis en "cargas 2026.xlsx"</t>
   </si>
   <si>
     <t xml:space="preserve">             cuando te equivocas. Separadas por punto y coma.</t>
@@ -707,25 +644,25 @@
     <t xml:space="preserve">             agregas aca y listo, no se toca codigo.</t>
   </si>
   <si>
-    <t xml:space="preserve">Pais       = Brasil / Paraguay / Bolivia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Region     = ej. Norte SC, Vale do Itajai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Municipio  = ej. Luiz Alves, Guaramirim  (con esto cruzo el clima)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Localidad  = barrio, comunidad o paraje. El detalle fino.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lat / Lon  = NO las llenes. Las completo yo a partir del municipio.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Km_acopio  = distancia al acopio, si la sabes. Opcional.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notas      = lo que quieras: calidad, forma de pago, lo que sea.</t>
+    <t>Pais       = Brasil / Paraguay / Bolivia</t>
+  </si>
+  <si>
+    <t>Region     = ej. Norte SC, Vale do Itajai</t>
+  </si>
+  <si>
+    <t>Municipio  = ej. Luiz Alves, Guaramirim  (con esto cruzo el clima)</t>
+  </si>
+  <si>
+    <t>Localidad  = barrio, comunidad o paraje. El detalle fino.</t>
+  </si>
+  <si>
+    <t>Lat / Lon  = NO las llenes. Las completo yo a partir del municipio.</t>
+  </si>
+  <si>
+    <t>Km_acopio  = distancia al acopio, si la sabes. Opcional.</t>
+  </si>
+  <si>
+    <t>Notas      = lo que quieras: calidad, forma de pago, lo que sea.</t>
   </si>
   <si>
     <t>Cargas_2026_ref = solo referencia, para que veas quien es grande y quien</t>
@@ -746,37 +683,37 @@
     <t>nombre del productor, en el ranking de "Real 2026 BR" del dashboard:</t>
   </si>
   <si>
-    <t xml:space="preserve">Nombre_completo  = nombre o razon social. Los que ya estan vienen de la</t>
+    <t>Nombre_completo  = nombre o razon social. Los que ya estan vienen de la</t>
   </si>
   <si>
     <t xml:space="preserve">                   planilla del Plan de Cargas; corregilos si hace falta.</t>
   </si>
   <si>
-    <t xml:space="preserve">Direccion        = calle / km / referencia de la finca o del packing.</t>
+    <t>Direccion        = calle / km / referencia de la finca o del packing.</t>
   </si>
   <si>
     <t>Hectareas_banana = hectareas plantadas con banana (numero, ej 12,5).</t>
   </si>
   <si>
-    <t xml:space="preserve">Pies_banana      = cantidad de pies / plantas (numero, ej 18000). Si</t>
+    <t>Pies_banana      = cantidad de pies / plantas (numero, ej 18000). Si</t>
   </si>
   <si>
     <t xml:space="preserve">                   estan los dos, la ficha calcula pies por hectarea.</t>
   </si>
   <si>
-    <t xml:space="preserve">Variedad         = Nanica, Prata, Grande Naine...</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Packing          = Propio / Tercero / Almar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Certificaciones  = GlobalGAP, organico, etc. Vacio si no tiene.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contacto         = telefono / WhatsApp. Es columna de texto, con +55.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Desde            = anio en que empezo a cargar para Almar.</t>
+    <t>Variedad         = Nanica, Prata, Grande Naine...</t>
+  </si>
+  <si>
+    <t>Packing          = Propio / Tercero / Almar.</t>
+  </si>
+  <si>
+    <t>Certificaciones  = GlobalGAP, organico, etc. Vacio si no tiene.</t>
+  </si>
+  <si>
+    <t>Contacto         = telefono / WhatsApp. Es columna de texto, con +55.</t>
+  </si>
+  <si>
+    <t>Desde            = anio en que empezo a cargar para Almar.</t>
   </si>
   <si>
     <t>Lat / Lon: si las cargas (decimales con signo, ej -26.72 / -48.93) la</t>
@@ -792,14 +729,16 @@
   </si>
   <si>
     <t>Lo que no llenes sale como "-" en la ficha. Nada se rompe por dejar vacio.</t>
+  </si>
+  <si>
+    <t>COMPRADOR, no productor: revende fruta de otros. En el Plan de Cargas sus camiones figuran con el nombre del productor real (Curuca solo aparece 2 veces, canceladas: 27/02 y 24/03/2026). Compras 2026: sem 5 con FG (carpeta BRB011-26) y sem 14-16 con Chabat/Etimex (carpetas BRB029-26, BRB035-26, BRB036-26); el vendedor exacto de cada camion esta en esas carpetas de Etimex.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -831,6 +770,20 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -866,19 +819,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="0" applyNumberFormat="1" fontId="2" applyFont="1" fillId="2" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="3" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="0" applyNumberFormat="1" fontId="3" applyFont="1" fillId="3" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" applyNumberFormat="1" fontId="3" applyFont="1" fillId="3" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1196,17 +1149,17 @@
   <dimension ref="A1:W26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" bestFit="1" width="14.28515625" customWidth="1"/>
+    <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="3" bestFit="1" width="9.140625" customWidth="1"/>
-    <col min="4" max="4" bestFit="1" width="11.7109375" customWidth="1"/>
-    <col min="5" max="5" bestFit="1" width="14.5703125" customWidth="1"/>
-    <col min="6" max="6" bestFit="1" width="13.85546875" customWidth="1"/>
-    <col min="7" max="7" bestFit="1" width="8.140625" customWidth="1"/>
-    <col min="8" max="8" bestFit="1" width="8.7109375" customWidth="1"/>
-    <col min="9" max="9" bestFit="1" width="15.28515625" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="30.7109375" customWidth="1"/>
-    <col min="11" max="11" bestFit="1" width="20.7109375" customWidth="1"/>
+    <col min="11" max="11" width="20.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="28.7109375" customWidth="1"/>
     <col min="13" max="13" width="34.7109375" customWidth="1"/>
     <col min="14" max="14" width="16.7109375" customWidth="1"/>
@@ -1214,11 +1167,11 @@
     <col min="16" max="16" width="14.7109375" customWidth="1"/>
     <col min="17" max="17" width="12.7109375" customWidth="1"/>
     <col min="18" max="18" width="18.7109375" customWidth="1"/>
-    <col min="19" max="19" width="20.7109375" customWidth="1" style="6"/>
-    <col min="20" max="20" width="8.7109375" customWidth="1" style="6"/>
+    <col min="19" max="19" width="20.7109375" style="6" customWidth="1"/>
+    <col min="20" max="20" width="8.7109375" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1289,535 +1242,505 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="0" t="s">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" t="s">
         <v>25</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" t="s">
         <v>27</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" t="s">
         <v>28</v>
       </c>
       <c r="G2" s="3">
-        <v>-26.3796942</v>
+        <v>-26.379694199999999</v>
       </c>
       <c r="H2" s="3">
-        <v>-49.2812341</v>
-      </c>
-      <c r="J2" s="0" t="s">
-        <v>29</v>
+        <v>-49.281234099999999</v>
       </c>
       <c r="K2" s="3">
         <v>95</v>
       </c>
-      <c r="L2" s="0" t="s">
+      <c r="L2" t="s">
         <v>24</v>
       </c>
-      <c r="M2" s="0" t="s">
+      <c r="M2" t="s">
+        <v>29</v>
+      </c>
+      <c r="P2" t="s">
         <v>30</v>
       </c>
-      <c r="P2" s="0" t="s">
+      <c r="S2" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="S2" s="6" t="s">
+      <c r="T2" s="6" t="s">
         <v>32</v>
-      </c>
-      <c r="T2" s="6" t="s">
-        <v>33</v>
       </c>
       <c r="U2" s="6"/>
       <c r="V2" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="W2" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="W2" s="6" t="s">
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="0" t="s">
+      <c r="B3" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="0" t="s">
-        <v>37</v>
-      </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" t="s">
         <v>25</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" t="s">
         <v>26</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" t="s">
         <v>27</v>
       </c>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
-      <c r="J3" s="0" t="s">
-        <v>29</v>
-      </c>
       <c r="K3" s="3">
         <v>61</v>
       </c>
-      <c r="L3" s="0" t="s">
+      <c r="L3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M3" t="s">
         <v>38</v>
       </c>
-      <c r="M3" s="0" t="s">
+      <c r="O3">
+        <v>200000</v>
+      </c>
+      <c r="P3" t="s">
+        <v>30</v>
+      </c>
+      <c r="S3" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="O3" s="0">
-        <v>200000</v>
-      </c>
-      <c r="P3" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="S3" s="6" t="s">
+      <c r="T3" s="6" t="s">
         <v>40</v>
-      </c>
-      <c r="T3" s="6" t="s">
-        <v>41</v>
       </c>
       <c r="U3" s="6"/>
       <c r="V3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="W3" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="W3" s="6" t="s">
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="0" t="s">
+      <c r="B4" t="s">
         <v>44</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" t="s">
         <v>45</v>
       </c>
-      <c r="C4" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="D4" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" s="0" t="s">
+      <c r="F4" t="s">
         <v>46</v>
       </c>
-      <c r="F4" s="0" t="s">
-        <v>47</v>
-      </c>
       <c r="G4" s="3">
-        <v>-26.677312</v>
+        <v>-26.677312000000001</v>
       </c>
       <c r="H4" s="3">
         <v>-48.893062</v>
       </c>
-      <c r="J4" s="0" t="s">
-        <v>48</v>
-      </c>
       <c r="K4" s="3">
         <v>34</v>
       </c>
-      <c r="L4" s="0" t="s">
+      <c r="L4" t="s">
+        <v>47</v>
+      </c>
+      <c r="M4" t="s">
+        <v>48</v>
+      </c>
+      <c r="P4" t="s">
+        <v>30</v>
+      </c>
+      <c r="S4" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="M4" s="0" t="s">
+      <c r="T4" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="P4" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="S4" s="6" t="s">
+      <c r="U4" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="T4" s="6" t="s">
+      <c r="V4" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="U4" s="6" t="s">
+      <c r="W4" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="V4" s="6" t="s">
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>54</v>
       </c>
-      <c r="W4" s="6" t="s">
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="C5" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" s="0" t="s">
-        <v>57</v>
-      </c>
       <c r="G5" s="3">
-        <v>-26.4961677</v>
+        <v>-26.496167700000001</v>
       </c>
       <c r="H5" s="3">
-        <v>-48.9038862</v>
-      </c>
-      <c r="J5" s="0" t="s">
-        <v>58</v>
+        <v>-48.903886200000002</v>
       </c>
       <c r="K5" s="3">
         <v>40.5</v>
       </c>
-      <c r="M5" s="0" t="s">
-        <v>59</v>
-      </c>
-      <c r="O5" s="0">
+      <c r="M5" t="s">
+        <v>56</v>
+      </c>
+      <c r="O5">
         <v>65000</v>
       </c>
-      <c r="P5" s="0" t="s">
-        <v>60</v>
+      <c r="P5" t="s">
+        <v>57</v>
       </c>
       <c r="S5" s="6" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="T5" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="U5" s="6"/>
       <c r="V5" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="W5" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" t="s">
         <v>62</v>
       </c>
-      <c r="W5" s="6" t="s">
+      <c r="C6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="0" t="s">
-        <v>64</v>
-      </c>
-      <c r="B6" s="0" t="s">
-        <v>65</v>
-      </c>
-      <c r="C6" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" s="0" t="s">
-        <v>66</v>
-      </c>
       <c r="G6" s="3">
-        <v>-26.685313</v>
+        <v>-26.685313000000001</v>
       </c>
       <c r="H6" s="3">
-        <v>-48.778437</v>
-      </c>
-      <c r="J6" s="0" t="s">
-        <v>67</v>
+        <v>-48.778436999999997</v>
       </c>
       <c r="K6" s="3">
         <v>26</v>
       </c>
-      <c r="L6" s="0" t="s">
+      <c r="L6" t="s">
+        <v>64</v>
+      </c>
+      <c r="M6" t="s">
+        <v>65</v>
+      </c>
+      <c r="P6" t="s">
+        <v>30</v>
+      </c>
+      <c r="T6" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="U6" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="V6" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="M6" s="0" t="s">
+      <c r="W6" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="P6" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="T6" s="6" t="s">
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>70</v>
       </c>
-      <c r="U6" s="6" t="s">
+      <c r="B7" t="s">
         <v>71</v>
       </c>
-      <c r="V6" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="W6" s="6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="0" t="s">
-        <v>74</v>
-      </c>
-      <c r="B7" s="0" t="s">
-        <v>75</v>
-      </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="0" t="s">
-        <v>46</v>
+      <c r="E7" t="s">
+        <v>45</v>
       </c>
       <c r="G7" s="3">
         <v>-26.6920769</v>
       </c>
       <c r="H7" s="3">
-        <v>-48.8342889</v>
-      </c>
-      <c r="J7" s="0" t="s">
-        <v>76</v>
+        <v>-48.834288899999997</v>
       </c>
       <c r="K7" s="3">
         <v>45.5</v>
       </c>
-      <c r="M7" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="P7" s="0" t="s">
-        <v>31</v>
+      <c r="M7" t="s">
+        <v>72</v>
+      </c>
+      <c r="P7" t="s">
+        <v>30</v>
       </c>
       <c r="T7" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="U7" s="6"/>
       <c r="V7" s="6" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="W7" s="6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="B8" s="0" t="s">
-        <v>80</v>
-      </c>
-      <c r="C8" s="0" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C8" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="0" t="s">
-        <v>81</v>
-      </c>
-      <c r="F8" s="0" t="s">
-        <v>82</v>
+      <c r="E8" t="s">
+        <v>76</v>
+      </c>
+      <c r="F8" t="s">
+        <v>77</v>
       </c>
       <c r="G8" s="3">
-        <v>-26.571301</v>
+        <v>-26.571300999999998</v>
       </c>
       <c r="H8" s="3">
-        <v>-48.8425407</v>
-      </c>
-      <c r="J8" s="0" t="s">
-        <v>83</v>
+        <v>-48.842540700000001</v>
       </c>
       <c r="K8" s="3">
         <v>19</v>
       </c>
-      <c r="L8" s="0" t="s">
-        <v>80</v>
-      </c>
-      <c r="P8" s="0" t="s">
-        <v>31</v>
+      <c r="L8" t="s">
+        <v>75</v>
+      </c>
+      <c r="P8" t="s">
+        <v>30</v>
       </c>
       <c r="S8" s="6" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="T8" s="6" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="U8" s="6"/>
       <c r="V8" s="6" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="W8" s="6" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="0" t="s">
-        <v>88</v>
-      </c>
-      <c r="B9" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="C9" s="0" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>82</v>
+      </c>
+      <c r="B9" t="s">
+        <v>83</v>
+      </c>
+      <c r="C9" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="0" t="s">
+      <c r="E9" t="s">
+        <v>45</v>
+      </c>
+      <c r="F9" t="s">
         <v>46</v>
       </c>
-      <c r="F9" s="0" t="s">
-        <v>47</v>
-      </c>
       <c r="G9" s="3">
-        <v>-26.6543969</v>
+        <v>-26.654396899999998</v>
       </c>
       <c r="H9" s="3">
-        <v>-48.880387</v>
-      </c>
-      <c r="J9" s="0" t="s">
-        <v>90</v>
+        <v>-48.880386999999999</v>
       </c>
       <c r="K9" s="3">
         <v>19.5</v>
       </c>
-      <c r="L9" s="0" t="s">
-        <v>91</v>
-      </c>
-      <c r="M9" s="0" t="s">
-        <v>92</v>
-      </c>
-      <c r="N9" s="0">
+      <c r="L9" t="s">
+        <v>84</v>
+      </c>
+      <c r="M9" t="s">
+        <v>85</v>
+      </c>
+      <c r="N9">
         <v>10</v>
       </c>
-      <c r="O9" s="0">
+      <c r="O9">
         <v>35000</v>
       </c>
-      <c r="P9" s="0" t="s">
-        <v>31</v>
+      <c r="P9" t="s">
+        <v>30</v>
       </c>
       <c r="S9" s="6" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="T9" s="6" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="U9" s="6"/>
       <c r="V9" s="6" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="W9" s="6" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="0" t="s">
-        <v>97</v>
-      </c>
-      <c r="B10" s="0" t="s">
-        <v>98</v>
-      </c>
-      <c r="C10" s="0" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B10" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="F10" s="0" t="s">
-        <v>99</v>
+      <c r="E10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" t="s">
+        <v>92</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
-      <c r="J10" s="0" t="s">
-        <v>29</v>
-      </c>
       <c r="K10" s="3">
         <v>14</v>
       </c>
-      <c r="L10" s="0" t="s">
-        <v>98</v>
-      </c>
-      <c r="M10" s="0" t="s">
-        <v>100</v>
-      </c>
-      <c r="O10" s="0">
+      <c r="L10" t="s">
+        <v>91</v>
+      </c>
+      <c r="M10" t="s">
+        <v>93</v>
+      </c>
+      <c r="O10">
         <v>40000</v>
       </c>
-      <c r="P10" s="0" t="s">
-        <v>31</v>
+      <c r="P10" t="s">
+        <v>30</v>
       </c>
       <c r="S10" s="6" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="T10" s="6" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="U10" s="6"/>
       <c r="V10" s="6" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="W10" s="6" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="0" t="s">
-        <v>105</v>
-      </c>
-      <c r="B11" s="0" t="s">
-        <v>106</v>
-      </c>
-      <c r="C11" s="0" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>98</v>
+      </c>
+      <c r="B11" t="s">
+        <v>99</v>
+      </c>
+      <c r="C11" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="D11" t="s">
         <v>26</v>
       </c>
-      <c r="E11" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="F11" s="0" t="s">
-        <v>107</v>
+      <c r="E11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" t="s">
+        <v>100</v>
       </c>
       <c r="G11" s="3">
-        <v>-26.71657</v>
+        <v>-26.716570000000001</v>
       </c>
       <c r="H11" s="3">
         <v>-48.836506</v>
       </c>
-      <c r="J11" s="0" t="s">
-        <v>108</v>
-      </c>
       <c r="K11" s="3">
         <v>12</v>
       </c>
-      <c r="L11" s="0" t="s">
-        <v>109</v>
-      </c>
-      <c r="P11" s="0" t="s">
-        <v>31</v>
+      <c r="L11" t="s">
+        <v>101</v>
+      </c>
+      <c r="P11" t="s">
+        <v>30</v>
       </c>
       <c r="S11" s="6" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="T11" s="6" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="U11" s="6"/>
       <c r="V11" s="6" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="W11" s="6" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="0" t="s">
-        <v>113</v>
-      </c>
-      <c r="B12" s="0" t="s">
-        <v>114</v>
-      </c>
-      <c r="C12" s="0" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>105</v>
+      </c>
+      <c r="B12" t="s">
+        <v>106</v>
+      </c>
+      <c r="C12" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" t="s">
         <v>26</v>
       </c>
       <c r="G12" s="3"/>
@@ -1825,548 +1748,508 @@
       <c r="K12" s="3">
         <v>6</v>
       </c>
-      <c r="L12" s="0" t="s">
-        <v>115</v>
-      </c>
-      <c r="P12" s="0" t="s">
-        <v>31</v>
+      <c r="L12" t="s">
+        <v>107</v>
+      </c>
+      <c r="P12" t="s">
+        <v>30</v>
       </c>
       <c r="T12" s="6" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="U12" s="6" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="V12" s="6"/>
       <c r="W12" s="6"/>
     </row>
-    <row r="13">
-      <c r="A13" s="0" t="s">
-        <v>117</v>
-      </c>
-      <c r="C13" s="0" t="s">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>109</v>
+      </c>
+      <c r="C13" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="0" t="s">
+      <c r="D13" t="s">
         <v>26</v>
       </c>
-      <c r="E13" s="0" t="s">
-        <v>118</v>
-      </c>
-      <c r="F13" s="0" t="s">
-        <v>119</v>
+      <c r="E13" t="s">
+        <v>110</v>
+      </c>
+      <c r="F13" t="s">
+        <v>111</v>
       </c>
       <c r="G13" s="3">
-        <v>-26.733688</v>
+        <v>-26.733688000000001</v>
       </c>
       <c r="H13" s="3">
-        <v>-48.768562</v>
-      </c>
-      <c r="J13" s="0" t="s">
-        <v>120</v>
+        <v>-48.768562000000003</v>
       </c>
       <c r="K13" s="3">
         <v>6</v>
       </c>
-      <c r="L13" s="0" t="s">
-        <v>121</v>
-      </c>
-      <c r="M13" s="0" t="s">
-        <v>122</v>
-      </c>
-      <c r="P13" s="0" t="s">
-        <v>31</v>
+      <c r="L13" t="s">
+        <v>112</v>
+      </c>
+      <c r="M13" t="s">
+        <v>113</v>
+      </c>
+      <c r="P13" t="s">
+        <v>30</v>
       </c>
       <c r="S13" s="6" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
       <c r="T13" s="6" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="U13" s="6" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="V13" s="6" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="W13" s="6" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="0" t="s">
-        <v>126</v>
-      </c>
-      <c r="C14" s="0" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>117</v>
+      </c>
+      <c r="C14" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="0" t="s">
+      <c r="D14" t="s">
         <v>26</v>
       </c>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
-      <c r="J14" s="0" t="s">
-        <v>127</v>
+      <c r="J14" t="s">
+        <v>216</v>
       </c>
       <c r="K14" s="3">
         <v>6</v>
       </c>
-      <c r="P14" s="0" t="s">
-        <v>31</v>
+      <c r="P14" t="s">
+        <v>30</v>
       </c>
       <c r="T14" s="6" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="U14" s="6" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="V14" s="6"/>
       <c r="W14" s="6"/>
     </row>
-    <row r="15">
-      <c r="A15" s="0" t="s">
-        <v>128</v>
-      </c>
-      <c r="B15" s="0" t="s">
-        <v>129</v>
-      </c>
-      <c r="C15" s="0" t="s">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>118</v>
+      </c>
+      <c r="B15" t="s">
+        <v>119</v>
+      </c>
+      <c r="C15" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="0" t="s">
+      <c r="D15" t="s">
         <v>26</v>
       </c>
-      <c r="E15" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="F15" s="0" t="s">
-        <v>131</v>
+      <c r="E15" t="s">
+        <v>120</v>
+      </c>
+      <c r="F15" t="s">
+        <v>121</v>
       </c>
       <c r="G15" s="3">
         <v>-26.709688</v>
       </c>
       <c r="H15" s="3">
-        <v>-48.794562</v>
-      </c>
-      <c r="J15" s="0" t="s">
-        <v>29</v>
+        <v>-48.794561999999999</v>
       </c>
       <c r="K15" s="3">
         <v>11.5</v>
       </c>
-      <c r="M15" s="0" t="s">
-        <v>132</v>
-      </c>
-      <c r="O15" s="0">
+      <c r="M15" t="s">
+        <v>122</v>
+      </c>
+      <c r="O15">
         <v>33000</v>
       </c>
-      <c r="P15" s="0" t="s">
-        <v>31</v>
+      <c r="P15" t="s">
+        <v>30</v>
       </c>
       <c r="S15" s="6" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="T15" s="6" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="U15" s="6"/>
       <c r="V15" s="6" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="W15" s="6" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="0" t="s">
-        <v>137</v>
-      </c>
-      <c r="B16" s="0" t="s">
-        <v>138</v>
-      </c>
-      <c r="C16" s="0" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>127</v>
+      </c>
+      <c r="B16" t="s">
+        <v>128</v>
+      </c>
+      <c r="C16" t="s">
         <v>25</v>
       </c>
-      <c r="D16" s="0" t="s">
+      <c r="D16" t="s">
         <v>26</v>
       </c>
-      <c r="E16" s="0" t="s">
-        <v>46</v>
+      <c r="E16" t="s">
+        <v>45</v>
       </c>
       <c r="G16" s="3">
-        <v>-26.667188</v>
+        <v>-26.667187999999999</v>
       </c>
       <c r="H16" s="3">
-        <v>-48.876062</v>
-      </c>
-      <c r="J16" s="0" t="s">
-        <v>139</v>
+        <v>-48.876061999999997</v>
       </c>
       <c r="K16" s="3">
         <v>17</v>
       </c>
-      <c r="L16" s="0" t="s">
-        <v>138</v>
-      </c>
-      <c r="M16" s="0" t="s">
-        <v>140</v>
-      </c>
-      <c r="O16" s="0">
+      <c r="L16" t="s">
+        <v>128</v>
+      </c>
+      <c r="M16" t="s">
+        <v>129</v>
+      </c>
+      <c r="O16">
         <v>85000</v>
       </c>
-      <c r="P16" s="0" t="s">
-        <v>31</v>
+      <c r="P16" t="s">
+        <v>30</v>
       </c>
       <c r="S16" s="6" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="T16" s="6" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="U16" s="6"/>
       <c r="V16" s="6" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="W16" s="6" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="0" t="s">
-        <v>144</v>
-      </c>
-      <c r="B17" s="0" t="s">
-        <v>145</v>
-      </c>
-      <c r="C17" s="0" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>133</v>
+      </c>
+      <c r="B17" t="s">
+        <v>134</v>
+      </c>
+      <c r="C17" t="s">
         <v>25</v>
       </c>
-      <c r="D17" s="0" t="s">
+      <c r="D17" t="s">
         <v>26</v>
       </c>
-      <c r="E17" s="0" t="s">
-        <v>66</v>
-      </c>
-      <c r="J17" s="0" t="s">
-        <v>146</v>
-      </c>
-      <c r="K17" s="0">
+      <c r="E17" t="s">
+        <v>63</v>
+      </c>
+      <c r="K17">
         <v>8</v>
       </c>
-      <c r="L17" s="0" t="s">
-        <v>145</v>
-      </c>
-      <c r="M17" s="0" t="s">
-        <v>147</v>
-      </c>
-      <c r="P17" s="0" t="s">
-        <v>31</v>
+      <c r="L17" t="s">
+        <v>134</v>
+      </c>
+      <c r="M17" t="s">
+        <v>135</v>
+      </c>
+      <c r="P17" t="s">
+        <v>30</v>
       </c>
       <c r="S17" s="6" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="T17" s="6" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="U17" s="6"/>
       <c r="V17" s="6" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="W17" s="6" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="0" t="s">
-        <v>152</v>
-      </c>
-      <c r="B18" s="0" t="s">
-        <v>153</v>
-      </c>
-      <c r="C18" s="0" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>140</v>
+      </c>
+      <c r="B18" t="s">
+        <v>141</v>
+      </c>
+      <c r="C18" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="0" t="s">
+      <c r="D18" t="s">
         <v>26</v>
       </c>
-      <c r="E18" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="F18" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="G18" s="0">
-        <v>-26.6724542</v>
-      </c>
-      <c r="H18" s="0">
-        <v>-48.9256154</v>
-      </c>
-      <c r="J18" s="0" t="s">
-        <v>155</v>
-      </c>
-      <c r="K18" s="0">
+      <c r="E18" t="s">
+        <v>45</v>
+      </c>
+      <c r="F18" t="s">
+        <v>142</v>
+      </c>
+      <c r="G18">
+        <v>-26.672454200000001</v>
+      </c>
+      <c r="H18">
+        <v>-48.925615399999998</v>
+      </c>
+      <c r="K18">
         <v>4</v>
       </c>
-      <c r="L18" s="0" t="s">
-        <v>156</v>
-      </c>
-      <c r="P18" s="0" t="s">
-        <v>31</v>
+      <c r="L18" t="s">
+        <v>143</v>
+      </c>
+      <c r="P18" t="s">
+        <v>30</v>
       </c>
       <c r="S18" s="6" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
       <c r="T18" s="6" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="U18" s="6"/>
       <c r="V18" s="6" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="W18" s="6" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="0" t="s">
-        <v>159</v>
-      </c>
-      <c r="C19" s="0" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>146</v>
+      </c>
+      <c r="C19" t="s">
         <v>25</v>
       </c>
-      <c r="D19" s="0" t="s">
+      <c r="D19" t="s">
         <v>26</v>
       </c>
-      <c r="E19" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="G19" s="0">
-        <v>-26.635688</v>
-      </c>
-      <c r="H19" s="0">
-        <v>-48.850312</v>
-      </c>
-      <c r="J19" s="0" t="s">
-        <v>160</v>
-      </c>
-      <c r="K19" s="0">
+      <c r="E19" t="s">
+        <v>45</v>
+      </c>
+      <c r="G19">
+        <v>-26.635687999999998</v>
+      </c>
+      <c r="H19">
+        <v>-48.850312000000002</v>
+      </c>
+      <c r="K19">
         <v>1.5</v>
       </c>
-      <c r="M19" s="0" t="s">
-        <v>161</v>
-      </c>
-      <c r="P19" s="0" t="s">
-        <v>31</v>
+      <c r="M19" t="s">
+        <v>147</v>
+      </c>
+      <c r="P19" t="s">
+        <v>30</v>
       </c>
       <c r="T19" s="6" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="U19" s="6"/>
       <c r="V19" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="W19" s="6" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>149</v>
+      </c>
+      <c r="B20" t="s">
+        <v>150</v>
+      </c>
+      <c r="C20" t="s">
+        <v>151</v>
+      </c>
+      <c r="D20" t="s">
+        <v>152</v>
+      </c>
+      <c r="E20" t="s">
+        <v>153</v>
+      </c>
+      <c r="G20">
+        <v>-25.3264</v>
+      </c>
+      <c r="H20">
+        <v>-55.372100000000003</v>
+      </c>
+      <c r="K20">
+        <v>65</v>
+      </c>
+      <c r="L20" t="s">
+        <v>154</v>
+      </c>
+      <c r="M20" t="s">
+        <v>155</v>
+      </c>
+      <c r="T20" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="V20">
+        <v>1388</v>
+      </c>
+      <c r="W20">
+        <v>1390</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>157</v>
+      </c>
+      <c r="B21" t="s">
+        <v>158</v>
+      </c>
+      <c r="C21" t="s">
+        <v>151</v>
+      </c>
+      <c r="D21" t="s">
+        <v>152</v>
+      </c>
+      <c r="G21">
+        <v>-25.344809999999999</v>
+      </c>
+      <c r="H21">
+        <v>-55.480310000000003</v>
+      </c>
+      <c r="K21">
+        <v>15</v>
+      </c>
+      <c r="L21" t="s">
+        <v>159</v>
+      </c>
+      <c r="M21" t="s">
+        <v>160</v>
+      </c>
+      <c r="T21" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="V21">
+        <v>1402</v>
+      </c>
+      <c r="W21">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>161</v>
+      </c>
+      <c r="B22" t="s">
         <v>162</v>
       </c>
-      <c r="W19" s="6" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="0" t="s">
+      <c r="C22" t="s">
+        <v>151</v>
+      </c>
+      <c r="K22">
+        <v>0</v>
+      </c>
+      <c r="T22" s="6" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>163</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B23" t="s">
         <v>164</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="C23" t="s">
+        <v>151</v>
+      </c>
+      <c r="K23">
+        <v>17</v>
+      </c>
+      <c r="L23" t="s">
         <v>165</v>
       </c>
-      <c r="D20" s="0" t="s">
+      <c r="T23" s="6" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>166</v>
       </c>
-      <c r="E20" s="0" t="s">
+      <c r="B24" t="s">
         <v>167</v>
       </c>
-      <c r="G20" s="0">
-        <v>-25.3264</v>
-      </c>
-      <c r="H20" s="0">
-        <v>-55.3721</v>
-      </c>
-      <c r="J20" s="0" t="s">
+      <c r="C24" t="s">
+        <v>151</v>
+      </c>
+      <c r="K24">
+        <v>11</v>
+      </c>
+      <c r="L24" t="s">
         <v>168</v>
       </c>
-      <c r="K20" s="0">
-        <v>65</v>
-      </c>
-      <c r="L20" s="0" t="s">
+      <c r="T24" s="6" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>169</v>
       </c>
-      <c r="M20" s="0" t="s">
+      <c r="B25" t="s">
         <v>170</v>
       </c>
-      <c r="T20" s="6" t="s">
+      <c r="C25" t="s">
+        <v>151</v>
+      </c>
+      <c r="K25">
+        <v>7</v>
+      </c>
+      <c r="L25" t="s">
         <v>171</v>
       </c>
-      <c r="V20" s="0">
-        <v>1388</v>
-      </c>
-      <c r="W20" s="0">
-        <v>1390</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="0" t="s">
+      <c r="T25" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="B21" s="0" t="s">
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>173</v>
       </c>
-      <c r="C21" s="0" t="s">
-        <v>165</v>
-      </c>
-      <c r="D21" s="0" t="s">
-        <v>166</v>
-      </c>
-      <c r="G21" s="0">
-        <v>-25.34481</v>
-      </c>
-      <c r="H21" s="0">
-        <v>-55.48031</v>
-      </c>
-      <c r="J21" s="0" t="s">
+      <c r="B26" t="s">
         <v>174</v>
       </c>
-      <c r="K21" s="0">
-        <v>15</v>
-      </c>
-      <c r="L21" s="0" t="s">
+      <c r="C26" t="s">
+        <v>151</v>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+      <c r="T26" s="6" t="s">
         <v>175</v>
-      </c>
-      <c r="M21" s="0" t="s">
-        <v>176</v>
-      </c>
-      <c r="T21" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="V21" s="0">
-        <v>1402</v>
-      </c>
-      <c r="W21" s="0">
-        <v>1404</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="B22" s="0" t="s">
-        <v>178</v>
-      </c>
-      <c r="C22" s="0" t="s">
-        <v>165</v>
-      </c>
-      <c r="J22" s="0" t="s">
-        <v>179</v>
-      </c>
-      <c r="K22" s="0">
-        <v>0</v>
-      </c>
-      <c r="T22" s="6" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="0" t="s">
-        <v>180</v>
-      </c>
-      <c r="B23" s="0" t="s">
-        <v>181</v>
-      </c>
-      <c r="C23" s="0" t="s">
-        <v>165</v>
-      </c>
-      <c r="J23" s="0" t="s">
-        <v>182</v>
-      </c>
-      <c r="K23" s="0">
-        <v>17</v>
-      </c>
-      <c r="L23" s="0" t="s">
-        <v>183</v>
-      </c>
-      <c r="T23" s="6" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="0" t="s">
-        <v>184</v>
-      </c>
-      <c r="B24" s="0" t="s">
-        <v>185</v>
-      </c>
-      <c r="C24" s="0" t="s">
-        <v>165</v>
-      </c>
-      <c r="J24" s="0" t="s">
-        <v>186</v>
-      </c>
-      <c r="K24" s="0">
-        <v>11</v>
-      </c>
-      <c r="L24" s="0" t="s">
-        <v>187</v>
-      </c>
-      <c r="T24" s="6" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="0" t="s">
-        <v>188</v>
-      </c>
-      <c r="B25" s="0" t="s">
-        <v>189</v>
-      </c>
-      <c r="C25" s="0" t="s">
-        <v>165</v>
-      </c>
-      <c r="J25" s="0" t="s">
-        <v>190</v>
-      </c>
-      <c r="K25" s="0">
-        <v>7</v>
-      </c>
-      <c r="L25" s="0" t="s">
-        <v>191</v>
-      </c>
-      <c r="T25" s="6" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="0" t="s">
-        <v>193</v>
-      </c>
-      <c r="B26" s="0" t="s">
-        <v>194</v>
-      </c>
-      <c r="C26" s="0" t="s">
-        <v>165</v>
-      </c>
-      <c r="J26" s="0" t="s">
-        <v>195</v>
-      </c>
-      <c r="K26" s="0">
-        <v>0</v>
-      </c>
-      <c r="T26" s="6" t="s">
-        <v>196</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K1" xr:uid="{AE80DDAC-136B-4211-BF28-F3220B5B0972}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -2379,208 +2262,207 @@
     <col min="1" max="1" width="78.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="0" t="s">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="0" t="s">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="0" t="s">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="0" t="s">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="0" t="s">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="0" t="s">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="0" t="s">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="0" t="s">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="0" t="s">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="0" t="s">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="0" t="s">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="0" t="s">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="0" t="s">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="0" t="s">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="0" t="s">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="0" t="s">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="0" t="s">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="0" t="s">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
         <v>215</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="0" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="0" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="0" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="0" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="0" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="0" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="0" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="0" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="0" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="0" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="0" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="0" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="0" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="0" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="0" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="0" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="0" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="0" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="0" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="0" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="0" t="s">
-        <v>236</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Alvarito (Paraguay AS): ubicacion de la finca en la ficha (Toro Piru, San Pedro, plus code 5875MHG3+PQ) y zona de clima py_toro_piru
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/productores.xlsx
+++ b/fuentes/productores.xlsx
@@ -17,9 +17,9 @@
     <sheet name="como_llenar" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">productores!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'productores'!$A$1:$K$1</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="220">
   <si>
     <t>Productor</t>
   </si>
@@ -437,6 +437,9 @@
     <t>Curuca</t>
   </si>
   <si>
+    <t>COMPRADOR, no productor: revende fruta de otros. En el Plan de Cargas sus camiones figuran con el nombre del productor real (Curuca solo aparece 2 veces, canceladas: 27/02 y 24/03/2026). Compras 2026: sem 5 con FG (carpeta BRB011-26) y sem 14-16 con Chabat/Etimex (carpetas BRB029-26, BRB035-26, BRB036-26); el vendedor exacto de cada camion esta en esas carpetas de Etimex.</t>
+  </si>
+  <si>
     <t>Furlani</t>
   </si>
   <si>
@@ -596,9 +599,18 @@
     <t>AS; PY AS</t>
   </si>
   <si>
+    <t>San Pedro</t>
+  </si>
+  <si>
+    <t>Toro Pirú</t>
+  </si>
+  <si>
     <t>Alvaro Saldivar</t>
   </si>
   <si>
+    <t>MHG3+PQC, Toro Pirú 021603, Paraguay (plus code 5875MHG3+PQ, Gonzalo 24/09/2026)</t>
+  </si>
+  <si>
     <t>ago 2026</t>
   </si>
   <si>
@@ -620,13 +632,13 @@
     <t>un productor nuevo o si cambia algo.</t>
   </si>
   <si>
-    <t>Productor  = nombre canonico. NO tocar los que ya estan: son los que el</t>
+    <t xml:space="preserve">Productor  = nombre canonico. NO tocar los que ya estan: son los que el</t>
   </si>
   <si>
     <t xml:space="preserve">             script ya reconoce.</t>
   </si>
   <si>
-    <t>Alias      = todas las formas en que lo escribis en "cargas 2026.xlsx"</t>
+    <t xml:space="preserve">Alias      = todas las formas en que lo escribis en "cargas 2026.xlsx"</t>
   </si>
   <si>
     <t xml:space="preserve">             cuando te equivocas. Separadas por punto y coma.</t>
@@ -644,25 +656,25 @@
     <t xml:space="preserve">             agregas aca y listo, no se toca codigo.</t>
   </si>
   <si>
-    <t>Pais       = Brasil / Paraguay / Bolivia</t>
-  </si>
-  <si>
-    <t>Region     = ej. Norte SC, Vale do Itajai</t>
-  </si>
-  <si>
-    <t>Municipio  = ej. Luiz Alves, Guaramirim  (con esto cruzo el clima)</t>
-  </si>
-  <si>
-    <t>Localidad  = barrio, comunidad o paraje. El detalle fino.</t>
-  </si>
-  <si>
-    <t>Lat / Lon  = NO las llenes. Las completo yo a partir del municipio.</t>
-  </si>
-  <si>
-    <t>Km_acopio  = distancia al acopio, si la sabes. Opcional.</t>
-  </si>
-  <si>
-    <t>Notas      = lo que quieras: calidad, forma de pago, lo que sea.</t>
+    <t xml:space="preserve">Pais       = Brasil / Paraguay / Bolivia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Region     = ej. Norte SC, Vale do Itajai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Municipio  = ej. Luiz Alves, Guaramirim  (con esto cruzo el clima)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Localidad  = barrio, comunidad o paraje. El detalle fino.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lat / Lon  = NO las llenes. Las completo yo a partir del municipio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Km_acopio  = distancia al acopio, si la sabes. Opcional.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notas      = lo que quieras: calidad, forma de pago, lo que sea.</t>
   </si>
   <si>
     <t>Cargas_2026_ref = solo referencia, para que veas quien es grande y quien</t>
@@ -683,37 +695,37 @@
     <t>nombre del productor, en el ranking de "Real 2026 BR" del dashboard:</t>
   </si>
   <si>
-    <t>Nombre_completo  = nombre o razon social. Los que ya estan vienen de la</t>
+    <t xml:space="preserve">Nombre_completo  = nombre o razon social. Los que ya estan vienen de la</t>
   </si>
   <si>
     <t xml:space="preserve">                   planilla del Plan de Cargas; corregilos si hace falta.</t>
   </si>
   <si>
-    <t>Direccion        = calle / km / referencia de la finca o del packing.</t>
+    <t xml:space="preserve">Direccion        = calle / km / referencia de la finca o del packing.</t>
   </si>
   <si>
     <t>Hectareas_banana = hectareas plantadas con banana (numero, ej 12,5).</t>
   </si>
   <si>
-    <t>Pies_banana      = cantidad de pies / plantas (numero, ej 18000). Si</t>
+    <t xml:space="preserve">Pies_banana      = cantidad de pies / plantas (numero, ej 18000). Si</t>
   </si>
   <si>
     <t xml:space="preserve">                   estan los dos, la ficha calcula pies por hectarea.</t>
   </si>
   <si>
-    <t>Variedad         = Nanica, Prata, Grande Naine...</t>
-  </si>
-  <si>
-    <t>Packing          = Propio / Tercero / Almar.</t>
-  </si>
-  <si>
-    <t>Certificaciones  = GlobalGAP, organico, etc. Vacio si no tiene.</t>
-  </si>
-  <si>
-    <t>Contacto         = telefono / WhatsApp. Es columna de texto, con +55.</t>
-  </si>
-  <si>
-    <t>Desde            = anio en que empezo a cargar para Almar.</t>
+    <t xml:space="preserve">Variedad         = Nanica, Prata, Grande Naine...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Packing          = Propio / Tercero / Almar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Certificaciones  = GlobalGAP, organico, etc. Vacio si no tiene.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contacto         = telefono / WhatsApp. Es columna de texto, con +55.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desde            = anio en que empezo a cargar para Almar.</t>
   </si>
   <si>
     <t>Lat / Lon: si las cargas (decimales con signo, ej -26.72 / -48.93) la</t>
@@ -729,16 +741,14 @@
   </si>
   <si>
     <t>Lo que no llenes sale como "-" en la ficha. Nada se rompe por dejar vacio.</t>
-  </si>
-  <si>
-    <t>COMPRADOR, no productor: revende fruta de otros. En el Plan de Cargas sus camiones figuran con el nombre del productor real (Curuca solo aparece 2 veces, canceladas: 27/02 y 24/03/2026). Compras 2026: sem 5 con FG (carpeta BRB011-26) y sem 14-16 con Chabat/Etimex (carpetas BRB029-26, BRB035-26, BRB036-26); el vendedor exacto de cada camion esta en esas carpetas de Etimex.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -770,20 +780,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -819,19 +815,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="2" applyFont="1" fillId="2" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="3" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="3" applyFont="1" fillId="3" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" applyNumberFormat="1" fontId="3" applyFont="1" fillId="3" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1149,17 +1145,17 @@
   <dimension ref="A1:W26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="1" width="14.28515625" customWidth="1"/>
     <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" bestFit="1" width="9.140625" customWidth="1"/>
+    <col min="4" max="4" bestFit="1" width="11.7109375" customWidth="1"/>
+    <col min="5" max="5" bestFit="1" width="14.5703125" customWidth="1"/>
+    <col min="6" max="6" bestFit="1" width="13.85546875" customWidth="1"/>
+    <col min="7" max="7" bestFit="1" width="8.140625" customWidth="1"/>
+    <col min="8" max="8" bestFit="1" width="8.7109375" customWidth="1"/>
+    <col min="9" max="9" bestFit="1" width="15.28515625" customWidth="1"/>
     <col min="10" max="10" width="30.7109375" customWidth="1"/>
-    <col min="11" max="11" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" bestFit="1" width="20.7109375" customWidth="1"/>
     <col min="12" max="12" width="28.7109375" customWidth="1"/>
     <col min="13" max="13" width="34.7109375" customWidth="1"/>
     <col min="14" max="14" width="16.7109375" customWidth="1"/>
@@ -1167,11 +1163,11 @@
     <col min="16" max="16" width="14.7109375" customWidth="1"/>
     <col min="17" max="17" width="12.7109375" customWidth="1"/>
     <col min="18" max="18" width="18.7109375" customWidth="1"/>
-    <col min="19" max="19" width="20.7109375" style="6" customWidth="1"/>
-    <col min="20" max="20" width="8.7109375" style="6" customWidth="1"/>
+    <col min="19" max="19" width="20.7109375" customWidth="1" style="6"/>
+    <col min="20" max="20" width="8.7109375" customWidth="1" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1242,41 +1238,41 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2">
+      <c r="A2" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="0" t="s">
         <v>28</v>
       </c>
       <c r="G2" s="3">
-        <v>-26.379694199999999</v>
+        <v>-26.3796942</v>
       </c>
       <c r="H2" s="3">
-        <v>-49.281234099999999</v>
+        <v>-49.2812341</v>
       </c>
       <c r="K2" s="3">
         <v>95</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="P2" t="s">
+      <c r="P2" s="0" t="s">
         <v>30</v>
       </c>
       <c r="S2" s="6" t="s">
@@ -1293,20 +1289,20 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3">
+      <c r="A3" s="0" t="s">
         <v>35</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="0" t="s">
         <v>36</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="0" t="s">
         <v>27</v>
       </c>
       <c r="G3" s="3"/>
@@ -1314,16 +1310,16 @@
       <c r="K3" s="3">
         <v>61</v>
       </c>
-      <c r="L3" t="s">
+      <c r="L3" s="0" t="s">
         <v>37</v>
       </c>
-      <c r="M3" t="s">
+      <c r="M3" s="0" t="s">
         <v>38</v>
       </c>
-      <c r="O3">
+      <c r="O3" s="0">
         <v>200000</v>
       </c>
-      <c r="P3" t="s">
+      <c r="P3" s="0" t="s">
         <v>30</v>
       </c>
       <c r="S3" s="6" t="s">
@@ -1340,27 +1336,27 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4">
+      <c r="A4" s="0" t="s">
         <v>43</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="0" t="s">
         <v>44</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="0" t="s">
         <v>45</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="0" t="s">
         <v>46</v>
       </c>
       <c r="G4" s="3">
-        <v>-26.677312000000001</v>
+        <v>-26.677312</v>
       </c>
       <c r="H4" s="3">
         <v>-48.893062</v>
@@ -1368,13 +1364,13 @@
       <c r="K4" s="3">
         <v>34</v>
       </c>
-      <c r="L4" t="s">
+      <c r="L4" s="0" t="s">
         <v>47</v>
       </c>
-      <c r="M4" t="s">
+      <c r="M4" s="0" t="s">
         <v>48</v>
       </c>
-      <c r="P4" t="s">
+      <c r="P4" s="0" t="s">
         <v>30</v>
       </c>
       <c r="S4" s="6" t="s">
@@ -1393,35 +1389,35 @@
         <v>53</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5">
+      <c r="A5" s="0" t="s">
         <v>54</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="0" t="s">
         <v>55</v>
       </c>
       <c r="G5" s="3">
-        <v>-26.496167700000001</v>
+        <v>-26.4961677</v>
       </c>
       <c r="H5" s="3">
-        <v>-48.903886200000002</v>
+        <v>-48.9038862</v>
       </c>
       <c r="K5" s="3">
         <v>40.5</v>
       </c>
-      <c r="M5" t="s">
+      <c r="M5" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="O5">
+      <c r="O5" s="0">
         <v>65000</v>
       </c>
-      <c r="P5" t="s">
+      <c r="P5" s="0" t="s">
         <v>57</v>
       </c>
       <c r="S5" s="6" t="s">
@@ -1438,38 +1434,38 @@
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6">
+      <c r="A6" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="0" t="s">
         <v>63</v>
       </c>
       <c r="G6" s="3">
-        <v>-26.685313000000001</v>
+        <v>-26.685313</v>
       </c>
       <c r="H6" s="3">
-        <v>-48.778436999999997</v>
+        <v>-48.778437</v>
       </c>
       <c r="K6" s="3">
         <v>26</v>
       </c>
-      <c r="L6" t="s">
+      <c r="L6" s="0" t="s">
         <v>64</v>
       </c>
-      <c r="M6" t="s">
+      <c r="M6" s="0" t="s">
         <v>65</v>
       </c>
-      <c r="P6" t="s">
+      <c r="P6" s="0" t="s">
         <v>30</v>
       </c>
       <c r="T6" s="6" t="s">
@@ -1485,35 +1481,35 @@
         <v>69</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7">
+      <c r="A7" s="0" t="s">
         <v>70</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="0" t="s">
         <v>45</v>
       </c>
       <c r="G7" s="3">
         <v>-26.6920769</v>
       </c>
       <c r="H7" s="3">
-        <v>-48.834288899999997</v>
+        <v>-48.8342889</v>
       </c>
       <c r="K7" s="3">
         <v>45.5</v>
       </c>
-      <c r="M7" t="s">
+      <c r="M7" s="0" t="s">
         <v>72</v>
       </c>
-      <c r="P7" t="s">
+      <c r="P7" s="0" t="s">
         <v>30</v>
       </c>
       <c r="T7" s="6" t="s">
@@ -1527,38 +1523,38 @@
         <v>73</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8">
+      <c r="A8" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="0" t="s">
         <v>76</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="0" t="s">
         <v>77</v>
       </c>
       <c r="G8" s="3">
-        <v>-26.571300999999998</v>
+        <v>-26.571301</v>
       </c>
       <c r="H8" s="3">
-        <v>-48.842540700000001</v>
+        <v>-48.8425407</v>
       </c>
       <c r="K8" s="3">
         <v>19</v>
       </c>
-      <c r="L8" t="s">
+      <c r="L8" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="P8" t="s">
+      <c r="P8" s="0" t="s">
         <v>30</v>
       </c>
       <c r="S8" s="6" t="s">
@@ -1575,47 +1571,47 @@
         <v>81</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="9">
+      <c r="A9" s="0" t="s">
         <v>82</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="0" t="s">
         <v>83</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="0" t="s">
         <v>45</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="0" t="s">
         <v>46</v>
       </c>
       <c r="G9" s="3">
-        <v>-26.654396899999998</v>
+        <v>-26.6543969</v>
       </c>
       <c r="H9" s="3">
-        <v>-48.880386999999999</v>
+        <v>-48.880387</v>
       </c>
       <c r="K9" s="3">
         <v>19.5</v>
       </c>
-      <c r="L9" t="s">
+      <c r="L9" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="M9" t="s">
+      <c r="M9" s="0" t="s">
         <v>85</v>
       </c>
-      <c r="N9">
+      <c r="N9" s="0">
         <v>10</v>
       </c>
-      <c r="O9">
+      <c r="O9" s="0">
         <v>35000</v>
       </c>
-      <c r="P9" t="s">
+      <c r="P9" s="0" t="s">
         <v>30</v>
       </c>
       <c r="S9" s="6" t="s">
@@ -1632,23 +1628,23 @@
         <v>89</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="10">
+      <c r="A10" s="0" t="s">
         <v>90</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="0" t="s">
         <v>91</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="0" t="s">
         <v>45</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="0" t="s">
         <v>92</v>
       </c>
       <c r="G10" s="3"/>
@@ -1656,16 +1652,16 @@
       <c r="K10" s="3">
         <v>14</v>
       </c>
-      <c r="L10" t="s">
+      <c r="L10" s="0" t="s">
         <v>91</v>
       </c>
-      <c r="M10" t="s">
+      <c r="M10" s="0" t="s">
         <v>93</v>
       </c>
-      <c r="O10">
+      <c r="O10" s="0">
         <v>40000</v>
       </c>
-      <c r="P10" t="s">
+      <c r="P10" s="0" t="s">
         <v>30</v>
       </c>
       <c r="S10" s="6" t="s">
@@ -1682,27 +1678,27 @@
         <v>97</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11">
+      <c r="A11" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="0" t="s">
         <v>45</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="0" t="s">
         <v>100</v>
       </c>
       <c r="G11" s="3">
-        <v>-26.716570000000001</v>
+        <v>-26.71657</v>
       </c>
       <c r="H11" s="3">
         <v>-48.836506</v>
@@ -1710,10 +1706,10 @@
       <c r="K11" s="3">
         <v>12</v>
       </c>
-      <c r="L11" t="s">
+      <c r="L11" s="0" t="s">
         <v>101</v>
       </c>
-      <c r="P11" t="s">
+      <c r="P11" s="0" t="s">
         <v>30</v>
       </c>
       <c r="S11" s="6" t="s">
@@ -1730,17 +1726,17 @@
         <v>104</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="12">
+      <c r="A12" s="0" t="s">
         <v>105</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="0" t="s">
         <v>106</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="0" t="s">
         <v>26</v>
       </c>
       <c r="G12" s="3"/>
@@ -1748,10 +1744,10 @@
       <c r="K12" s="3">
         <v>6</v>
       </c>
-      <c r="L12" t="s">
+      <c r="L12" s="0" t="s">
         <v>107</v>
       </c>
-      <c r="P12" t="s">
+      <c r="P12" s="0" t="s">
         <v>30</v>
       </c>
       <c r="T12" s="6" t="s">
@@ -1763,38 +1759,38 @@
       <c r="V12" s="6"/>
       <c r="W12" s="6"/>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="13">
+      <c r="A13" s="0" t="s">
         <v>109</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="0" t="s">
         <v>110</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="0" t="s">
         <v>111</v>
       </c>
       <c r="G13" s="3">
-        <v>-26.733688000000001</v>
+        <v>-26.733688</v>
       </c>
       <c r="H13" s="3">
-        <v>-48.768562000000003</v>
+        <v>-48.768562</v>
       </c>
       <c r="K13" s="3">
         <v>6</v>
       </c>
-      <c r="L13" t="s">
+      <c r="L13" s="0" t="s">
         <v>112</v>
       </c>
-      <c r="M13" t="s">
+      <c r="M13" s="0" t="s">
         <v>113</v>
       </c>
-      <c r="P13" t="s">
+      <c r="P13" s="0" t="s">
         <v>30</v>
       </c>
       <c r="S13" s="6" t="s">
@@ -1813,25 +1809,25 @@
         <v>116</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="14">
+      <c r="A14" s="0" t="s">
         <v>117</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="0" t="s">
         <v>26</v>
       </c>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
-      <c r="J14" t="s">
-        <v>216</v>
+      <c r="J14" s="0" t="s">
+        <v>118</v>
       </c>
       <c r="K14" s="3">
         <v>6</v>
       </c>
-      <c r="P14" t="s">
+      <c r="P14" s="0" t="s">
         <v>30</v>
       </c>
       <c r="T14" s="6" t="s">
@@ -1843,413 +1839,429 @@
       <c r="V14" s="6"/>
       <c r="W14" s="6"/>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>118</v>
-      </c>
-      <c r="B15" t="s">
+    <row r="15">
+      <c r="A15" s="0" t="s">
         <v>119</v>
       </c>
-      <c r="C15" t="s">
+      <c r="B15" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="C15" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="E15" t="s">
-        <v>120</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="E15" s="0" t="s">
         <v>121</v>
+      </c>
+      <c r="F15" s="0" t="s">
+        <v>122</v>
       </c>
       <c r="G15" s="3">
         <v>-26.709688</v>
       </c>
       <c r="H15" s="3">
-        <v>-48.794561999999999</v>
+        <v>-48.794562</v>
       </c>
       <c r="K15" s="3">
         <v>11.5</v>
       </c>
-      <c r="M15" t="s">
-        <v>122</v>
-      </c>
-      <c r="O15">
+      <c r="M15" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="O15" s="0">
         <v>33000</v>
       </c>
-      <c r="P15" t="s">
+      <c r="P15" s="0" t="s">
         <v>30</v>
       </c>
       <c r="S15" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="T15" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="U15" s="6"/>
       <c r="V15" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="W15" s="6" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
         <v>127</v>
       </c>
-      <c r="B16" t="s">
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="s">
         <v>128</v>
       </c>
-      <c r="C16" t="s">
+      <c r="B16" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="C16" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="0" t="s">
         <v>45</v>
       </c>
       <c r="G16" s="3">
-        <v>-26.667187999999999</v>
+        <v>-26.667188</v>
       </c>
       <c r="H16" s="3">
-        <v>-48.876061999999997</v>
+        <v>-48.876062</v>
       </c>
       <c r="K16" s="3">
         <v>17</v>
       </c>
-      <c r="L16" t="s">
-        <v>128</v>
-      </c>
-      <c r="M16" t="s">
+      <c r="L16" s="0" t="s">
         <v>129</v>
       </c>
-      <c r="O16">
+      <c r="M16" s="0" t="s">
+        <v>130</v>
+      </c>
+      <c r="O16" s="0">
         <v>85000</v>
       </c>
-      <c r="P16" t="s">
+      <c r="P16" s="0" t="s">
         <v>30</v>
       </c>
       <c r="S16" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="T16" s="6" t="s">
         <v>87</v>
       </c>
       <c r="U16" s="6"/>
       <c r="V16" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="W16" s="6" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
         <v>133</v>
       </c>
-      <c r="B17" t="s">
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C17" t="s">
+      <c r="B17" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="C17" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="0" t="s">
         <v>63</v>
       </c>
-      <c r="K17">
+      <c r="K17" s="0">
         <v>8</v>
       </c>
-      <c r="L17" t="s">
-        <v>134</v>
-      </c>
-      <c r="M17" t="s">
+      <c r="L17" s="0" t="s">
         <v>135</v>
       </c>
-      <c r="P17" t="s">
+      <c r="M17" s="0" t="s">
+        <v>136</v>
+      </c>
+      <c r="P17" s="0" t="s">
         <v>30</v>
       </c>
       <c r="S17" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="T17" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="U17" s="6"/>
       <c r="V17" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="W17" s="6" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="B18" s="0" t="s">
+        <v>142</v>
+      </c>
+      <c r="C18" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="E18" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="F18" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="G18" s="0">
+        <v>-26.6724542</v>
+      </c>
+      <c r="H18" s="0">
+        <v>-48.9256154</v>
+      </c>
+      <c r="K18" s="0">
+        <v>4</v>
+      </c>
+      <c r="L18" s="0" t="s">
+        <v>144</v>
+      </c>
+      <c r="P18" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="S18" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="T18" s="6" t="s">
         <v>138</v>
-      </c>
-      <c r="W17" s="6" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>140</v>
-      </c>
-      <c r="B18" t="s">
-        <v>141</v>
-      </c>
-      <c r="C18" t="s">
-        <v>25</v>
-      </c>
-      <c r="D18" t="s">
-        <v>26</v>
-      </c>
-      <c r="E18" t="s">
-        <v>45</v>
-      </c>
-      <c r="F18" t="s">
-        <v>142</v>
-      </c>
-      <c r="G18">
-        <v>-26.672454200000001</v>
-      </c>
-      <c r="H18">
-        <v>-48.925615399999998</v>
-      </c>
-      <c r="K18">
-        <v>4</v>
-      </c>
-      <c r="L18" t="s">
-        <v>143</v>
-      </c>
-      <c r="P18" t="s">
-        <v>30</v>
-      </c>
-      <c r="S18" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="T18" s="6" t="s">
-        <v>137</v>
       </c>
       <c r="U18" s="6"/>
       <c r="V18" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="W18" s="6" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
         <v>146</v>
       </c>
-      <c r="C19" t="s">
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="C19" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="0" t="s">
         <v>45</v>
       </c>
-      <c r="G19">
-        <v>-26.635687999999998</v>
-      </c>
-      <c r="H19">
-        <v>-48.850312000000002</v>
-      </c>
-      <c r="K19">
+      <c r="G19" s="0">
+        <v>-26.635688</v>
+      </c>
+      <c r="H19" s="0">
+        <v>-48.850312</v>
+      </c>
+      <c r="K19" s="0">
         <v>1.5</v>
       </c>
-      <c r="M19" t="s">
-        <v>147</v>
-      </c>
-      <c r="P19" t="s">
+      <c r="M19" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="P19" s="0" t="s">
         <v>30</v>
       </c>
       <c r="T19" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="U19" s="6"/>
       <c r="V19" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="W19" s="6" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>149</v>
-      </c>
-      <c r="B20" t="s">
+    <row r="20">
+      <c r="A20" s="0" t="s">
         <v>150</v>
       </c>
-      <c r="C20" t="s">
+      <c r="B20" s="0" t="s">
         <v>151</v>
       </c>
-      <c r="D20" t="s">
+      <c r="C20" s="0" t="s">
         <v>152</v>
       </c>
-      <c r="E20" t="s">
+      <c r="D20" s="0" t="s">
         <v>153</v>
       </c>
-      <c r="G20">
+      <c r="E20" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="G20" s="0">
         <v>-25.3264</v>
       </c>
-      <c r="H20">
-        <v>-55.372100000000003</v>
-      </c>
-      <c r="K20">
+      <c r="H20" s="0">
+        <v>-55.3721</v>
+      </c>
+      <c r="K20" s="0">
         <v>65</v>
       </c>
-      <c r="L20" t="s">
-        <v>154</v>
-      </c>
-      <c r="M20" t="s">
+      <c r="L20" s="0" t="s">
         <v>155</v>
       </c>
+      <c r="M20" s="0" t="s">
+        <v>156</v>
+      </c>
       <c r="T20" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="V20">
+        <v>157</v>
+      </c>
+      <c r="V20" s="0">
         <v>1388</v>
       </c>
-      <c r="W20">
+      <c r="W20" s="0">
         <v>1390</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="21">
+      <c r="A21" s="0" t="s">
+        <v>158</v>
+      </c>
+      <c r="B21" s="0" t="s">
+        <v>159</v>
+      </c>
+      <c r="C21" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D21" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="G21" s="0">
+        <v>-25.34481</v>
+      </c>
+      <c r="H21" s="0">
+        <v>-55.48031</v>
+      </c>
+      <c r="K21" s="0">
+        <v>15</v>
+      </c>
+      <c r="L21" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="M21" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="T21" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="B21" t="s">
-        <v>158</v>
-      </c>
-      <c r="C21" t="s">
-        <v>151</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="V21" s="0">
+        <v>1402</v>
+      </c>
+      <c r="W21" s="0">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="s">
+        <v>162</v>
+      </c>
+      <c r="B22" s="0" t="s">
+        <v>163</v>
+      </c>
+      <c r="C22" s="0" t="s">
         <v>152</v>
       </c>
-      <c r="G21">
-        <v>-25.344809999999999</v>
-      </c>
-      <c r="H21">
-        <v>-55.480310000000003</v>
-      </c>
-      <c r="K21">
-        <v>15</v>
-      </c>
-      <c r="L21" t="s">
-        <v>159</v>
-      </c>
-      <c r="M21" t="s">
-        <v>160</v>
-      </c>
-      <c r="T21" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="V21">
-        <v>1402</v>
-      </c>
-      <c r="W21">
-        <v>1404</v>
-      </c>
-    </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>161</v>
-      </c>
-      <c r="B22" t="s">
-        <v>162</v>
-      </c>
-      <c r="C22" t="s">
-        <v>151</v>
-      </c>
-      <c r="K22">
+      <c r="K22" s="0">
         <v>0</v>
       </c>
       <c r="T22" s="6" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>163</v>
-      </c>
-      <c r="B23" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="s">
         <v>164</v>
       </c>
-      <c r="C23" t="s">
-        <v>151</v>
-      </c>
-      <c r="K23">
+      <c r="B23" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="C23" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="K23" s="0">
         <v>17</v>
       </c>
-      <c r="L23" t="s">
-        <v>165</v>
+      <c r="L23" s="0" t="s">
+        <v>166</v>
       </c>
       <c r="T23" s="6" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>166</v>
-      </c>
-      <c r="B24" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="s">
         <v>167</v>
       </c>
-      <c r="C24" t="s">
-        <v>151</v>
-      </c>
-      <c r="K24">
+      <c r="B24" s="0" t="s">
+        <v>168</v>
+      </c>
+      <c r="C24" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="K24" s="0">
         <v>11</v>
       </c>
-      <c r="L24" t="s">
-        <v>168</v>
+      <c r="L24" s="0" t="s">
+        <v>169</v>
       </c>
       <c r="T24" s="6" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>169</v>
-      </c>
-      <c r="B25" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="s">
         <v>170</v>
       </c>
-      <c r="C25" t="s">
-        <v>151</v>
-      </c>
-      <c r="K25">
+      <c r="B25" s="0" t="s">
+        <v>171</v>
+      </c>
+      <c r="C25" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D25" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="F25" s="0" t="s">
+        <v>173</v>
+      </c>
+      <c r="G25" s="0">
+        <v>-24.32306</v>
+      </c>
+      <c r="H25" s="0">
+        <v>-56.44544</v>
+      </c>
+      <c r="K25" s="0">
         <v>7</v>
       </c>
-      <c r="L25" t="s">
-        <v>171</v>
+      <c r="L25" s="0" t="s">
+        <v>174</v>
+      </c>
+      <c r="M25" s="0" t="s">
+        <v>175</v>
       </c>
       <c r="T25" s="6" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>173</v>
-      </c>
-      <c r="B26" t="s">
-        <v>174</v>
-      </c>
-      <c r="C26" t="s">
-        <v>151</v>
-      </c>
-      <c r="K26">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="s">
+        <v>177</v>
+      </c>
+      <c r="B26" s="0" t="s">
+        <v>178</v>
+      </c>
+      <c r="C26" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="K26" s="0">
         <v>0</v>
       </c>
       <c r="T26" s="6" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K1" xr:uid="{AE80DDAC-136B-4211-BF28-F3220B5B0972}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -2262,207 +2274,208 @@
     <col min="1" max="1" width="78.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" s="1" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="3">
+      <c r="A3" s="0" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="4">
+      <c r="A4" s="0" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="6">
+      <c r="A6" s="0" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="7">
+      <c r="A7" s="0" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="9">
+      <c r="A9" s="0" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="10">
+      <c r="A10" s="0" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="11">
+      <c r="A11" s="0" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="12">
+      <c r="A12" s="0" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="13">
+      <c r="A13" s="0" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="14">
+      <c r="A14" s="0" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="16">
+      <c r="A16" s="0" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="17">
+      <c r="A17" s="0" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="18">
+      <c r="A18" s="0" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="19">
+      <c r="A19" s="0" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="21">
+      <c r="A21" s="0" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="22">
+      <c r="A22" s="0" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="23">
+      <c r="A23" s="0" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row r="25">
+      <c r="A25" s="0" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row r="26">
+      <c r="A26" s="0" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+    <row r="27">
+      <c r="A27" s="0" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+    <row r="29">
+      <c r="A29" s="0" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+    <row r="31">
+      <c r="A31" s="0" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+    <row r="32">
+      <c r="A32" s="0" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+    <row r="34">
+      <c r="A34" s="0" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+    <row r="35">
+      <c r="A35" s="0" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+    <row r="36">
+      <c r="A36" s="0" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+    <row r="37">
+      <c r="A37" s="0" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+    <row r="38">
+      <c r="A38" s="0" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+    <row r="39">
+      <c r="A39" s="0" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+    <row r="40">
+      <c r="A40" s="0" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+    <row r="41">
+      <c r="A41" s="0" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+    <row r="42">
+      <c r="A42" s="0" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
+    <row r="43">
+      <c r="A43" s="0" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
+    <row r="44">
+      <c r="A44" s="0" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
+    <row r="46">
+      <c r="A46" s="0" t="s">
         <v>215</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="0" t="s">
+        <v>219</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fichas: fotos y videos de packing de EC, Alvarito, Milciades y HF (reproductor de video en la galeria); ubicacion de EC (Oga Lata, San Pedro) y GM (Mayor Otano, sin coordenadas)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/productores.xlsx
+++ b/fuentes/productores.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="228">
   <si>
     <t>Productor</t>
   </si>
@@ -575,6 +575,21 @@
     <t>EC; PY EC</t>
   </si>
   <si>
+    <t>San Pedro</t>
+  </si>
+  <si>
+    <t>Yrybucuá</t>
+  </si>
+  <si>
+    <t>Asent. Oga Lata</t>
+  </si>
+  <si>
+    <t>Banana EC</t>
+  </si>
+  <si>
+    <t>Unnamed Road, Asent. Oga Lata 021902, Paraguay (plus code GR6G+W3 = 5875GR6G+W3, Gonzalo 24/09/2026)</t>
+  </si>
+  <si>
     <t>Paraguay DF</t>
   </si>
   <si>
@@ -590,16 +605,25 @@
     <t>GM; PY GM</t>
   </si>
   <si>
-    <t>Servi Fel (Servifel)</t>
+    <t>Itapúa</t>
+  </si>
+  <si>
+    <t>Mayor Otaño</t>
+  </si>
+  <si>
+    <t>Zapallo</t>
+  </si>
+  <si>
+    <t>Guido · Servi Fel (Servifel)</t>
+  </si>
+  <si>
+    <t>Mayor Otaño 071806, Paraguay (plus code MH5P+JF Zapallo, Gonzalo 24/09/2026; ese codigo no cae en Paraguay, coordenadas pendientes)</t>
   </si>
   <si>
     <t>Paraguay AS</t>
   </si>
   <si>
     <t>AS; PY AS</t>
-  </si>
-  <si>
-    <t>San Pedro</t>
   </si>
   <si>
     <t>Toro Pirú</t>
@@ -2159,19 +2183,40 @@
       <c r="C22" s="0" t="s">
         <v>152</v>
       </c>
+      <c r="D22" s="0" t="s">
+        <v>164</v>
+      </c>
+      <c r="E22" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="F22" s="0" t="s">
+        <v>166</v>
+      </c>
+      <c r="G22" s="0">
+        <v>-24.48756</v>
+      </c>
+      <c r="H22" s="0">
+        <v>-56.12481</v>
+      </c>
       <c r="K22" s="0">
         <v>0</v>
       </c>
+      <c r="L22" s="0" t="s">
+        <v>167</v>
+      </c>
+      <c r="M22" s="0" t="s">
+        <v>168</v>
+      </c>
       <c r="T22" s="6" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="C23" s="0" t="s">
         <v>152</v>
@@ -2180,7 +2225,7 @@
         <v>17</v>
       </c>
       <c r="L23" s="0" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="T23" s="6" t="s">
         <v>157</v>
@@ -2188,19 +2233,31 @@
     </row>
     <row r="24">
       <c r="A24" s="0" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="C24" s="0" t="s">
         <v>152</v>
       </c>
+      <c r="D24" s="0" t="s">
+        <v>174</v>
+      </c>
+      <c r="E24" s="0" t="s">
+        <v>175</v>
+      </c>
+      <c r="F24" s="0" t="s">
+        <v>176</v>
+      </c>
       <c r="K24" s="0">
         <v>11</v>
       </c>
       <c r="L24" s="0" t="s">
-        <v>169</v>
+        <v>177</v>
+      </c>
+      <c r="M24" s="0" t="s">
+        <v>178</v>
       </c>
       <c r="T24" s="6" t="s">
         <v>157</v>
@@ -2208,19 +2265,19 @@
     </row>
     <row r="25">
       <c r="A25" s="0" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="C25" s="0" t="s">
         <v>152</v>
       </c>
       <c r="D25" s="0" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="G25" s="0">
         <v>-24.32306</v>
@@ -2232,21 +2289,21 @@
         <v>7</v>
       </c>
       <c r="L25" s="0" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="M25" s="0" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="T25" s="6" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="C26" s="0" t="s">
         <v>152</v>
@@ -2255,7 +2312,7 @@
         <v>0</v>
       </c>
       <c r="T26" s="6" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -2276,202 +2333,202 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="0" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="0" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="0" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="0" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="0" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="0" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="0" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="0" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="0" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="0" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="0" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="0" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="0" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="0" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="0" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="0" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Brasil: Curuca fuera del ranking (hoja reasignaciones -> productor real), Resumen ejecutivo abajo de Real BR, competencia con el formato de Penta (donas U VNA por anio, totales y tabla); paneles regenerados 21:10
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/productores.xlsx
+++ b/fuentes/productores.xlsx
@@ -15,6 +15,7 @@
   <sheets>
     <sheet name="productores" sheetId="1" r:id="rId1"/>
     <sheet name="como_llenar" sheetId="2" r:id="rId2"/>
+    <sheet name="reasignaciones" sheetId="3" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'productores'!$A$1:$K$1</definedName>
@@ -81,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="242">
   <si>
     <t>Productor</t>
   </si>
@@ -765,6 +766,48 @@
   </si>
   <si>
     <t>Lo que no llenes sale como "-" en la ficha. Nada se rompe por dejar vacio.</t>
+  </si>
+  <si>
+    <t>comprador</t>
+  </si>
+  <si>
+    <t>mes</t>
+  </si>
+  <si>
+    <t>semana</t>
+  </si>
+  <si>
+    <t>productor_real</t>
+  </si>
+  <si>
+    <t>cargas</t>
+  </si>
+  <si>
+    <t>nota</t>
+  </si>
+  <si>
+    <t>Enero</t>
+  </si>
+  <si>
+    <t>sem 26-31/01, R$ 30, Nilton; Plan: Marconi Kons 30/01 BRB013-26 (confirmado por Gonzalo 26/09)</t>
+  </si>
+  <si>
+    <t>Abril</t>
+  </si>
+  <si>
+    <t>sem 30/03-04/04, R$ 46, Chabat; Plan: Jorge Marangoni 03/04 BRB035-26</t>
+  </si>
+  <si>
+    <t>sem 30/03-04/04, R$ 46, Chabat; Plan: Wagner Schveitzer 04/04 BRB035-26</t>
+  </si>
+  <si>
+    <t>sem 06-11/04, R$ 39, Chabat; Plan: Jorge Marangoni 10/04 BRB036-26</t>
+  </si>
+  <si>
+    <t>sem 06-11/04, R$ 39, Chabat; Plan: Wagner Schveitzer 10/04 BRB036-26</t>
+  </si>
+  <si>
+    <t>sem 13-18/04, R$ 37, Chabat; Plan: Furlani 15/04 BRB036-26 (confirmado por Gonzalo 26/09)</t>
   </si>
 </sst>
 </file>
@@ -2535,4 +2578,162 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11.128748893737793" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" customWidth="1"/>
+    <col min="4" max="4" width="14.6583251953125" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" customWidth="1"/>
+    <col min="6" max="6" width="88.50623321533203" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>228</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>229</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>230</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>231</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>232</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>234</v>
+      </c>
+      <c r="C2" s="0">
+        <v>5</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="E2" s="0">
+        <v>1</v>
+      </c>
+      <c r="F2" s="0" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>236</v>
+      </c>
+      <c r="C3" s="0">
+        <v>14</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="E3" s="0">
+        <v>1</v>
+      </c>
+      <c r="F3" s="0" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>236</v>
+      </c>
+      <c r="C4" s="0">
+        <v>14</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="E4" s="0">
+        <v>1</v>
+      </c>
+      <c r="F4" s="0" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>236</v>
+      </c>
+      <c r="C5" s="0">
+        <v>15</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="E5" s="0">
+        <v>1</v>
+      </c>
+      <c r="F5" s="0" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>236</v>
+      </c>
+      <c r="C6" s="0">
+        <v>15</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="E6" s="0">
+        <v>1</v>
+      </c>
+      <c r="F6" s="0" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>236</v>
+      </c>
+      <c r="C7" s="0">
+        <v>16</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="E7" s="0">
+        <v>1</v>
+      </c>
+      <c r="F7" s="0" t="s">
+        <v>241</v>
+      </c>
+    </row>
+  </sheetData>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>